<commit_message>
Registra en la bitácora el SUS simulado que salió del postest de dos retiros.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/instrumentos/sesion-08/Sesion 8.xlsx
+++ b/instrumentos/sesion-08/Sesion 8.xlsx
@@ -27,9 +27,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
-    <numFmt numFmtId="165" formatCode="DD/MM/YYYY"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="DD/MM/YYYY"/>
   </numFmts>
   <fonts count="4">
     <font>
@@ -99,7 +98,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
@@ -108,8 +107,9 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="2" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="2" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="2" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -953,7 +953,7 @@
       <c r="A5" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="B5" s="4" t="n">
+      <c r="B5" s="6" t="n">
         <v>46321</v>
       </c>
       <c r="C5" s="3" t="inlineStr">
@@ -1011,7 +1011,7 @@
       <c r="A6" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="B6" s="4" t="n">
+      <c r="B6" s="6" t="n">
         <v>46321</v>
       </c>
       <c r="C6" s="3" t="inlineStr">
@@ -1069,7 +1069,7 @@
       <c r="A7" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="B7" s="4" t="n">
+      <c r="B7" s="6" t="n">
         <v>46321</v>
       </c>
       <c r="C7" s="3" t="inlineStr">
@@ -1094,7 +1094,7 @@
       </c>
       <c r="G7" s="3" t="inlineStr">
         <is>
-          <t>INCLUIR = 0 y sin postest. Los otros 105 quedan en 1</t>
+          <t>INCLUIR = 0 y sin postest. Los otros 105 quedan en 1 GU-TDH-015 y GU-TDH-033 tenían un SUS simulado de 82.5; salió de la columna de postest porque no rinden O2. Ese valor queda en esta bitácora.</t>
         </is>
       </c>
       <c r="H7" s="3" t="inlineStr">
@@ -1533,7 +1533,7 @@
       <c r="F5" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="G5" s="4" t="n">
+      <c r="G5" s="6" t="n">
         <v>46310</v>
       </c>
       <c r="H5" s="3" t="n">
@@ -1626,7 +1626,7 @@
       <c r="F6" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="G6" s="4" t="n">
+      <c r="G6" s="6" t="n">
         <v>46307</v>
       </c>
       <c r="H6" s="3" t="n">
@@ -1719,7 +1719,7 @@
       <c r="F7" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="G7" s="4" t="n">
+      <c r="G7" s="6" t="n">
         <v>46308</v>
       </c>
       <c r="H7" s="3" t="n">
@@ -1812,7 +1812,7 @@
       <c r="F8" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="G8" s="4" t="n">
+      <c r="G8" s="6" t="n">
         <v>46311</v>
       </c>
       <c r="H8" s="3" t="n">
@@ -1905,7 +1905,7 @@
       <c r="F9" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="G9" s="4" t="n">
+      <c r="G9" s="6" t="n">
         <v>46308</v>
       </c>
       <c r="H9" s="3" t="n">
@@ -1998,7 +1998,7 @@
       <c r="F10" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="G10" s="4" t="n">
+      <c r="G10" s="6" t="n">
         <v>46308</v>
       </c>
       <c r="H10" s="3" t="n">
@@ -2091,7 +2091,7 @@
       <c r="F11" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="G11" s="4" t="n">
+      <c r="G11" s="6" t="n">
         <v>46312</v>
       </c>
       <c r="H11" s="3" t="n">
@@ -2184,7 +2184,7 @@
       <c r="F12" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="G12" s="4" t="n">
+      <c r="G12" s="6" t="n">
         <v>46309</v>
       </c>
       <c r="H12" s="3" t="n">
@@ -2277,7 +2277,7 @@
       <c r="F13" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="G13" s="4" t="n">
+      <c r="G13" s="6" t="n">
         <v>46309</v>
       </c>
       <c r="H13" s="3" t="n">
@@ -2370,7 +2370,7 @@
       <c r="F14" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="G14" s="4" t="n">
+      <c r="G14" s="6" t="n">
         <v>46310</v>
       </c>
       <c r="H14" s="3" t="n">
@@ -2463,7 +2463,7 @@
       <c r="F15" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="G15" s="4" t="n">
+      <c r="G15" s="6" t="n">
         <v>46307</v>
       </c>
       <c r="H15" s="3" t="n">
@@ -2556,7 +2556,7 @@
       <c r="F16" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="G16" s="4" t="n">
+      <c r="G16" s="6" t="n">
         <v>46311</v>
       </c>
       <c r="H16" s="3" t="n">
@@ -2649,7 +2649,7 @@
       <c r="F17" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="G17" s="4" t="n">
+      <c r="G17" s="6" t="n">
         <v>46309</v>
       </c>
       <c r="H17" s="3" t="n">
@@ -2742,7 +2742,7 @@
       <c r="F18" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="G18" s="4" t="n">
+      <c r="G18" s="6" t="n">
         <v>46309</v>
       </c>
       <c r="H18" s="3" t="n">
@@ -2835,7 +2835,7 @@
       <c r="F19" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="G19" s="4" t="n">
+      <c r="G19" s="6" t="n">
         <v>46308</v>
       </c>
       <c r="H19" s="3" t="n">
@@ -2928,7 +2928,7 @@
       <c r="F20" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="G20" s="4" t="n">
+      <c r="G20" s="6" t="n">
         <v>46310</v>
       </c>
       <c r="H20" s="3" t="n">
@@ -3021,7 +3021,7 @@
       <c r="F21" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="G21" s="4" t="n">
+      <c r="G21" s="6" t="n">
         <v>46307</v>
       </c>
       <c r="H21" s="3" t="n">
@@ -3114,7 +3114,7 @@
       <c r="F22" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="G22" s="4" t="n">
+      <c r="G22" s="6" t="n">
         <v>46311</v>
       </c>
       <c r="H22" s="3" t="n">
@@ -3207,7 +3207,7 @@
       <c r="F23" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="G23" s="4" t="n">
+      <c r="G23" s="6" t="n">
         <v>46311</v>
       </c>
       <c r="H23" s="3" t="n">
@@ -3300,7 +3300,7 @@
       <c r="F24" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="G24" s="4" t="n">
+      <c r="G24" s="6" t="n">
         <v>46311</v>
       </c>
       <c r="H24" s="3" t="n">
@@ -3393,7 +3393,7 @@
       <c r="F25" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="G25" s="4" t="n">
+      <c r="G25" s="6" t="n">
         <v>46313</v>
       </c>
       <c r="H25" s="3" t="n">
@@ -3486,7 +3486,7 @@
       <c r="F26" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="G26" s="4" t="n">
+      <c r="G26" s="6" t="n">
         <v>46313</v>
       </c>
       <c r="H26" s="3" t="n">
@@ -3579,7 +3579,7 @@
       <c r="F27" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="G27" s="4" t="n">
+      <c r="G27" s="6" t="n">
         <v>46311</v>
       </c>
       <c r="H27" s="3" t="n">
@@ -3672,7 +3672,7 @@
       <c r="F28" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="G28" s="4" t="n">
+      <c r="G28" s="6" t="n">
         <v>46308</v>
       </c>
       <c r="H28" s="3" t="n">
@@ -3765,7 +3765,7 @@
       <c r="F29" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="G29" s="4" t="n">
+      <c r="G29" s="6" t="n">
         <v>46308</v>
       </c>
       <c r="H29" s="3" t="n">
@@ -3858,7 +3858,7 @@
       <c r="F30" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="G30" s="4" t="n">
+      <c r="G30" s="6" t="n">
         <v>46308</v>
       </c>
       <c r="H30" s="3" t="n">
@@ -3951,7 +3951,7 @@
       <c r="F31" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="G31" s="4" t="n">
+      <c r="G31" s="6" t="n">
         <v>46313</v>
       </c>
       <c r="H31" s="3" t="n">
@@ -4044,7 +4044,7 @@
       <c r="F32" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="G32" s="4" t="n">
+      <c r="G32" s="6" t="n">
         <v>46313</v>
       </c>
       <c r="H32" s="3" t="n">
@@ -4137,7 +4137,7 @@
       <c r="F33" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="G33" s="4" t="n">
+      <c r="G33" s="6" t="n">
         <v>46310</v>
       </c>
       <c r="H33" s="3" t="n">
@@ -4230,7 +4230,7 @@
       <c r="F34" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="G34" s="4" t="n">
+      <c r="G34" s="6" t="n">
         <v>46313</v>
       </c>
       <c r="H34" s="3" t="n">
@@ -4323,7 +4323,7 @@
       <c r="F35" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="G35" s="4" t="n">
+      <c r="G35" s="6" t="n">
         <v>46309</v>
       </c>
       <c r="H35" s="3" t="n">
@@ -4416,7 +4416,7 @@
       <c r="F36" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="G36" s="4" t="n">
+      <c r="G36" s="6" t="n">
         <v>46311</v>
       </c>
       <c r="H36" s="3" t="n">
@@ -4509,7 +4509,7 @@
       <c r="F37" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="G37" s="4" t="n">
+      <c r="G37" s="6" t="n">
         <v>46311</v>
       </c>
       <c r="H37" s="3" t="n">
@@ -4602,7 +4602,7 @@
       <c r="F38" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="G38" s="4" t="n">
+      <c r="G38" s="6" t="n">
         <v>46312</v>
       </c>
       <c r="H38" s="3" t="n">
@@ -4695,7 +4695,7 @@
       <c r="F39" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="G39" s="4" t="n">
+      <c r="G39" s="6" t="n">
         <v>46313</v>
       </c>
       <c r="H39" s="3" t="n">
@@ -4788,7 +4788,7 @@
       <c r="F40" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="G40" s="4" t="n">
+      <c r="G40" s="6" t="n">
         <v>46308</v>
       </c>
       <c r="H40" s="3" t="n">
@@ -4881,7 +4881,7 @@
       <c r="F41" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="G41" s="4" t="n">
+      <c r="G41" s="6" t="n">
         <v>46309</v>
       </c>
       <c r="H41" s="3" t="n">
@@ -4974,7 +4974,7 @@
       <c r="F42" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="G42" s="4" t="n">
+      <c r="G42" s="6" t="n">
         <v>46309</v>
       </c>
       <c r="H42" s="3" t="n">
@@ -5067,7 +5067,7 @@
       <c r="F43" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="G43" s="4" t="n">
+      <c r="G43" s="6" t="n">
         <v>46311</v>
       </c>
       <c r="H43" s="3" t="n">
@@ -5160,7 +5160,7 @@
       <c r="F44" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="G44" s="4" t="n">
+      <c r="G44" s="6" t="n">
         <v>46311</v>
       </c>
       <c r="H44" s="3" t="n">
@@ -5253,7 +5253,7 @@
       <c r="F45" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="G45" s="4" t="n">
+      <c r="G45" s="6" t="n">
         <v>46308</v>
       </c>
       <c r="H45" s="3" t="n">
@@ -5346,7 +5346,7 @@
       <c r="F46" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="G46" s="4" t="n">
+      <c r="G46" s="6" t="n">
         <v>46310</v>
       </c>
       <c r="H46" s="3" t="n">
@@ -5439,7 +5439,7 @@
       <c r="F47" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="G47" s="4" t="n">
+      <c r="G47" s="6" t="n">
         <v>46312</v>
       </c>
       <c r="H47" s="3" t="n">
@@ -5532,7 +5532,7 @@
       <c r="F48" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="G48" s="4" t="n">
+      <c r="G48" s="6" t="n">
         <v>46310</v>
       </c>
       <c r="H48" s="3" t="n">
@@ -5625,7 +5625,7 @@
       <c r="F49" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="G49" s="4" t="n">
+      <c r="G49" s="6" t="n">
         <v>46311</v>
       </c>
       <c r="H49" s="3" t="n">
@@ -5718,7 +5718,7 @@
       <c r="F50" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="G50" s="4" t="n">
+      <c r="G50" s="6" t="n">
         <v>46311</v>
       </c>
       <c r="H50" s="3" t="n">
@@ -5811,7 +5811,7 @@
       <c r="F51" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="G51" s="4" t="n">
+      <c r="G51" s="6" t="n">
         <v>46311</v>
       </c>
       <c r="H51" s="3" t="n">
@@ -5904,7 +5904,7 @@
       <c r="F52" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="G52" s="4" t="n">
+      <c r="G52" s="6" t="n">
         <v>46307</v>
       </c>
       <c r="H52" s="3" t="n">
@@ -5997,7 +5997,7 @@
       <c r="F53" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="G53" s="4" t="n">
+      <c r="G53" s="6" t="n">
         <v>46308</v>
       </c>
       <c r="H53" s="3" t="n">
@@ -6090,7 +6090,7 @@
       <c r="F54" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="G54" s="4" t="n">
+      <c r="G54" s="6" t="n">
         <v>46311</v>
       </c>
       <c r="H54" s="3" t="n">
@@ -6183,7 +6183,7 @@
       <c r="F55" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="G55" s="4" t="n">
+      <c r="G55" s="6" t="n">
         <v>46309</v>
       </c>
       <c r="H55" s="3" t="n">
@@ -6276,7 +6276,7 @@
       <c r="F56" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="G56" s="4" t="n">
+      <c r="G56" s="6" t="n">
         <v>46308</v>
       </c>
       <c r="H56" s="3" t="n">
@@ -6369,7 +6369,7 @@
       <c r="F57" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="G57" s="4" t="n">
+      <c r="G57" s="6" t="n">
         <v>46309</v>
       </c>
       <c r="H57" s="3" t="n">
@@ -6462,7 +6462,7 @@
       <c r="F58" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="G58" s="4" t="n">
+      <c r="G58" s="6" t="n">
         <v>46312</v>
       </c>
       <c r="H58" s="3" t="n">
@@ -6555,7 +6555,7 @@
       <c r="F59" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="G59" s="4" t="n">
+      <c r="G59" s="6" t="n">
         <v>46312</v>
       </c>
       <c r="H59" s="3" t="n">
@@ -6648,7 +6648,7 @@
       <c r="F60" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="G60" s="4" t="n">
+      <c r="G60" s="6" t="n">
         <v>46310</v>
       </c>
       <c r="H60" s="3" t="n">
@@ -6741,7 +6741,7 @@
       <c r="F61" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="G61" s="4" t="n">
+      <c r="G61" s="6" t="n">
         <v>46309</v>
       </c>
       <c r="H61" s="3" t="n">
@@ -6834,7 +6834,7 @@
       <c r="F62" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="G62" s="4" t="n">
+      <c r="G62" s="6" t="n">
         <v>46310</v>
       </c>
       <c r="H62" s="3" t="n">
@@ -6927,7 +6927,7 @@
       <c r="F63" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="G63" s="4" t="n">
+      <c r="G63" s="6" t="n">
         <v>46311</v>
       </c>
       <c r="H63" s="3" t="n">
@@ -7020,7 +7020,7 @@
       <c r="F64" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="G64" s="4" t="n">
+      <c r="G64" s="6" t="n">
         <v>46312</v>
       </c>
       <c r="H64" s="3" t="n">
@@ -7113,7 +7113,7 @@
       <c r="F65" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="G65" s="4" t="n">
+      <c r="G65" s="6" t="n">
         <v>46313</v>
       </c>
       <c r="H65" s="3" t="n">
@@ -7206,7 +7206,7 @@
       <c r="F66" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="G66" s="4" t="n">
+      <c r="G66" s="6" t="n">
         <v>46311</v>
       </c>
       <c r="H66" s="3" t="n">
@@ -7299,7 +7299,7 @@
       <c r="F67" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="G67" s="4" t="n">
+      <c r="G67" s="6" t="n">
         <v>46310</v>
       </c>
       <c r="H67" s="3" t="n">
@@ -7392,7 +7392,7 @@
       <c r="F68" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="G68" s="4" t="n">
+      <c r="G68" s="6" t="n">
         <v>46308</v>
       </c>
       <c r="H68" s="3" t="n">
@@ -7485,7 +7485,7 @@
       <c r="F69" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="G69" s="4" t="n">
+      <c r="G69" s="6" t="n">
         <v>46311</v>
       </c>
       <c r="H69" s="3" t="n">
@@ -7578,7 +7578,7 @@
       <c r="F70" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="G70" s="4" t="n">
+      <c r="G70" s="6" t="n">
         <v>46312</v>
       </c>
       <c r="H70" s="3" t="n">
@@ -7671,7 +7671,7 @@
       <c r="F71" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="G71" s="4" t="n">
+      <c r="G71" s="6" t="n">
         <v>46310</v>
       </c>
       <c r="H71" s="3" t="n">
@@ -7764,7 +7764,7 @@
       <c r="F72" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="G72" s="4" t="n">
+      <c r="G72" s="6" t="n">
         <v>46310</v>
       </c>
       <c r="H72" s="3" t="n">
@@ -7857,7 +7857,7 @@
       <c r="F73" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="G73" s="4" t="n">
+      <c r="G73" s="6" t="n">
         <v>46308</v>
       </c>
       <c r="H73" s="3" t="n">
@@ -7950,7 +7950,7 @@
       <c r="F74" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="G74" s="4" t="n">
+      <c r="G74" s="6" t="n">
         <v>46312</v>
       </c>
       <c r="H74" s="3" t="n">
@@ -8043,7 +8043,7 @@
       <c r="F75" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="G75" s="4" t="n">
+      <c r="G75" s="6" t="n">
         <v>46311</v>
       </c>
       <c r="H75" s="3" t="n">
@@ -8136,7 +8136,7 @@
       <c r="F76" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="G76" s="4" t="n">
+      <c r="G76" s="6" t="n">
         <v>46313</v>
       </c>
       <c r="H76" s="3" t="n">
@@ -8229,7 +8229,7 @@
       <c r="F77" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="G77" s="4" t="n">
+      <c r="G77" s="6" t="n">
         <v>46312</v>
       </c>
       <c r="H77" s="3" t="n">
@@ -8322,7 +8322,7 @@
       <c r="F78" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="G78" s="4" t="n">
+      <c r="G78" s="6" t="n">
         <v>46307</v>
       </c>
       <c r="H78" s="3" t="n">
@@ -8415,7 +8415,7 @@
       <c r="F79" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="G79" s="4" t="n">
+      <c r="G79" s="6" t="n">
         <v>46307</v>
       </c>
       <c r="H79" s="3" t="n">
@@ -8508,7 +8508,7 @@
       <c r="F80" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="G80" s="4" t="n">
+      <c r="G80" s="6" t="n">
         <v>46309</v>
       </c>
       <c r="H80" s="3" t="n">
@@ -8601,7 +8601,7 @@
       <c r="F81" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="G81" s="4" t="n">
+      <c r="G81" s="6" t="n">
         <v>46310</v>
       </c>
       <c r="H81" s="3" t="n">
@@ -8694,7 +8694,7 @@
       <c r="F82" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="G82" s="4" t="n">
+      <c r="G82" s="6" t="n">
         <v>46307</v>
       </c>
       <c r="H82" s="3" t="n">
@@ -8787,7 +8787,7 @@
       <c r="F83" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="G83" s="4" t="n">
+      <c r="G83" s="6" t="n">
         <v>46308</v>
       </c>
       <c r="H83" s="3" t="n">
@@ -8880,7 +8880,7 @@
       <c r="F84" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="G84" s="4" t="n">
+      <c r="G84" s="6" t="n">
         <v>46308</v>
       </c>
       <c r="H84" s="3" t="n">
@@ -8973,7 +8973,7 @@
       <c r="F85" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="G85" s="4" t="n">
+      <c r="G85" s="6" t="n">
         <v>46311</v>
       </c>
       <c r="H85" s="3" t="n">
@@ -9066,7 +9066,7 @@
       <c r="F86" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="G86" s="4" t="n">
+      <c r="G86" s="6" t="n">
         <v>46310</v>
       </c>
       <c r="H86" s="3" t="n">
@@ -9159,7 +9159,7 @@
       <c r="F87" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="G87" s="4" t="n">
+      <c r="G87" s="6" t="n">
         <v>46308</v>
       </c>
       <c r="H87" s="3" t="n">
@@ -9252,7 +9252,7 @@
       <c r="F88" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="G88" s="4" t="n">
+      <c r="G88" s="6" t="n">
         <v>46309</v>
       </c>
       <c r="H88" s="3" t="n">
@@ -9345,7 +9345,7 @@
       <c r="F89" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="G89" s="4" t="n">
+      <c r="G89" s="6" t="n">
         <v>46312</v>
       </c>
       <c r="H89" s="3" t="n">
@@ -9438,7 +9438,7 @@
       <c r="F90" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="G90" s="4" t="n">
+      <c r="G90" s="6" t="n">
         <v>46309</v>
       </c>
       <c r="H90" s="3" t="n">
@@ -9531,7 +9531,7 @@
       <c r="F91" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="G91" s="4" t="n">
+      <c r="G91" s="6" t="n">
         <v>46310</v>
       </c>
       <c r="H91" s="3" t="n">
@@ -9624,7 +9624,7 @@
       <c r="F92" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="G92" s="4" t="n">
+      <c r="G92" s="6" t="n">
         <v>46310</v>
       </c>
       <c r="H92" s="3" t="n">
@@ -9717,7 +9717,7 @@
       <c r="F93" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="G93" s="4" t="n">
+      <c r="G93" s="6" t="n">
         <v>46312</v>
       </c>
       <c r="H93" s="3" t="n">
@@ -9810,7 +9810,7 @@
       <c r="F94" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="G94" s="4" t="n">
+      <c r="G94" s="6" t="n">
         <v>46314</v>
       </c>
       <c r="H94" s="3" t="n">
@@ -9903,7 +9903,7 @@
       <c r="F95" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="G95" s="4" t="n">
+      <c r="G95" s="6" t="n">
         <v>46314</v>
       </c>
       <c r="H95" s="3" t="n">
@@ -9996,7 +9996,7 @@
       <c r="F96" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="G96" s="4" t="n">
+      <c r="G96" s="6" t="n">
         <v>46311</v>
       </c>
       <c r="H96" s="3" t="n">
@@ -10089,7 +10089,7 @@
       <c r="F97" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="G97" s="4" t="n">
+      <c r="G97" s="6" t="n">
         <v>46313</v>
       </c>
       <c r="H97" s="3" t="n">
@@ -10182,7 +10182,7 @@
       <c r="F98" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="G98" s="4" t="n">
+      <c r="G98" s="6" t="n">
         <v>46307</v>
       </c>
       <c r="H98" s="3" t="n">
@@ -10275,7 +10275,7 @@
       <c r="F99" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="G99" s="4" t="n">
+      <c r="G99" s="6" t="n">
         <v>46313</v>
       </c>
       <c r="H99" s="3" t="n">
@@ -10368,7 +10368,7 @@
       <c r="F100" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="G100" s="4" t="n">
+      <c r="G100" s="6" t="n">
         <v>46312</v>
       </c>
       <c r="H100" s="3" t="n">
@@ -10461,7 +10461,7 @@
       <c r="F101" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="G101" s="4" t="n">
+      <c r="G101" s="6" t="n">
         <v>46309</v>
       </c>
       <c r="H101" s="3" t="n">
@@ -10554,7 +10554,7 @@
       <c r="F102" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="G102" s="4" t="n">
+      <c r="G102" s="6" t="n">
         <v>46313</v>
       </c>
       <c r="H102" s="3" t="n">
@@ -10647,7 +10647,7 @@
       <c r="F103" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="G103" s="4" t="n">
+      <c r="G103" s="6" t="n">
         <v>46312</v>
       </c>
       <c r="H103" s="3" t="n">
@@ -10740,7 +10740,7 @@
       <c r="F104" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="G104" s="4" t="n">
+      <c r="G104" s="6" t="n">
         <v>46308</v>
       </c>
       <c r="H104" s="3" t="n">
@@ -10833,7 +10833,7 @@
       <c r="F105" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="G105" s="4" t="n">
+      <c r="G105" s="6" t="n">
         <v>46310</v>
       </c>
       <c r="H105" s="3" t="n">
@@ -10926,7 +10926,7 @@
       <c r="F106" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="G106" s="4" t="n">
+      <c r="G106" s="6" t="n">
         <v>46309</v>
       </c>
       <c r="H106" s="3" t="n">
@@ -11019,7 +11019,7 @@
       <c r="F107" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="G107" s="4" t="n">
+      <c r="G107" s="6" t="n">
         <v>46310</v>
       </c>
       <c r="H107" s="3" t="n">
@@ -11112,7 +11112,7 @@
       <c r="F108" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="G108" s="4" t="n">
+      <c r="G108" s="6" t="n">
         <v>46312</v>
       </c>
       <c r="H108" s="3" t="n">
@@ -11205,7 +11205,7 @@
       <c r="F109" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="G109" s="4" t="n">
+      <c r="G109" s="6" t="n">
         <v>46312</v>
       </c>
       <c r="H109" s="3" t="n">
@@ -11298,7 +11298,7 @@
       <c r="F110" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="G110" s="4" t="n">
+      <c r="G110" s="6" t="n">
         <v>46309</v>
       </c>
       <c r="H110" s="3" t="n">
@@ -11391,7 +11391,7 @@
       <c r="F111" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="G111" s="4" t="n">
+      <c r="G111" s="6" t="n">
         <v>46312</v>
       </c>
       <c r="H111" s="3" t="n">
@@ -11484,7 +11484,7 @@
       <c r="F112" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="G112" s="4" t="n">
+      <c r="G112" s="6" t="n">
         <v>46310</v>
       </c>
       <c r="H112" s="3" t="n">
@@ -11621,7 +11621,7 @@
           <t>GE</t>
         </is>
       </c>
-      <c r="C5" s="4" t="n">
+      <c r="C5" s="6" t="n">
         <v>46322</v>
       </c>
       <c r="D5" s="3" t="n">
@@ -11644,7 +11644,7 @@
           <t>GE</t>
         </is>
       </c>
-      <c r="C6" s="4" t="n">
+      <c r="C6" s="6" t="n">
         <v>46321</v>
       </c>
       <c r="D6" s="3" t="n">
@@ -11667,7 +11667,7 @@
           <t>GE</t>
         </is>
       </c>
-      <c r="C7" s="4" t="n">
+      <c r="C7" s="6" t="n">
         <v>46321</v>
       </c>
       <c r="D7" s="3" t="n">
@@ -11690,7 +11690,7 @@
           <t>GE</t>
         </is>
       </c>
-      <c r="C8" s="4" t="n">
+      <c r="C8" s="6" t="n">
         <v>46324</v>
       </c>
       <c r="D8" s="3" t="n">
@@ -11713,7 +11713,7 @@
           <t>GE</t>
         </is>
       </c>
-      <c r="C9" s="4" t="n">
+      <c r="C9" s="6" t="n">
         <v>46321</v>
       </c>
       <c r="D9" s="3" t="n">
@@ -11736,7 +11736,7 @@
           <t>GE</t>
         </is>
       </c>
-      <c r="C10" s="4" t="n">
+      <c r="C10" s="6" t="n">
         <v>46322</v>
       </c>
       <c r="D10" s="3" t="n">
@@ -11759,7 +11759,7 @@
           <t>GE</t>
         </is>
       </c>
-      <c r="C11" s="4" t="n">
+      <c r="C11" s="6" t="n">
         <v>46324</v>
       </c>
       <c r="D11" s="3" t="n">
@@ -11782,7 +11782,7 @@
           <t>GE</t>
         </is>
       </c>
-      <c r="C12" s="4" t="n">
+      <c r="C12" s="6" t="n">
         <v>46321</v>
       </c>
       <c r="D12" s="3" t="n">
@@ -11805,7 +11805,7 @@
           <t>GE</t>
         </is>
       </c>
-      <c r="C13" s="4" t="n">
+      <c r="C13" s="6" t="n">
         <v>46322</v>
       </c>
       <c r="D13" s="3" t="n">
@@ -11828,7 +11828,7 @@
           <t>GE</t>
         </is>
       </c>
-      <c r="C14" s="4" t="n">
+      <c r="C14" s="6" t="n">
         <v>46322</v>
       </c>
       <c r="D14" s="3" t="n">
@@ -11851,7 +11851,7 @@
           <t>GE</t>
         </is>
       </c>
-      <c r="C15" s="4" t="n">
+      <c r="C15" s="6" t="n">
         <v>46321</v>
       </c>
       <c r="D15" s="3" t="n">
@@ -11874,7 +11874,7 @@
           <t>GE</t>
         </is>
       </c>
-      <c r="C16" s="4" t="n">
+      <c r="C16" s="6" t="n">
         <v>46322</v>
       </c>
       <c r="D16" s="3" t="n">
@@ -11897,7 +11897,7 @@
           <t>GE</t>
         </is>
       </c>
-      <c r="C17" s="4" t="n">
+      <c r="C17" s="6" t="n">
         <v>46322</v>
       </c>
       <c r="D17" s="3" t="n">
@@ -11920,7 +11920,7 @@
           <t>GE</t>
         </is>
       </c>
-      <c r="C18" s="4" t="n">
+      <c r="C18" s="6" t="n">
         <v>46321</v>
       </c>
       <c r="D18" s="3" t="n">
@@ -11943,7 +11943,7 @@
           <t>GE</t>
         </is>
       </c>
-      <c r="C19" s="4" t="n">
+      <c r="C19" s="6" t="n">
         <v>46323</v>
       </c>
       <c r="D19" s="3" t="n">
@@ -11966,7 +11966,7 @@
           <t>GE</t>
         </is>
       </c>
-      <c r="C20" s="4" t="n">
+      <c r="C20" s="6" t="n">
         <v>46321</v>
       </c>
       <c r="D20" s="3" t="n">
@@ -11989,7 +11989,7 @@
           <t>GE</t>
         </is>
       </c>
-      <c r="C21" s="4" t="n">
+      <c r="C21" s="6" t="n">
         <v>46323</v>
       </c>
       <c r="D21" s="3" t="n">
@@ -12012,7 +12012,7 @@
           <t>GE</t>
         </is>
       </c>
-      <c r="C22" s="4" t="n">
+      <c r="C22" s="6" t="n">
         <v>46325</v>
       </c>
       <c r="D22" s="3" t="n">
@@ -12035,7 +12035,7 @@
           <t>GE</t>
         </is>
       </c>
-      <c r="C23" s="4" t="n">
+      <c r="C23" s="6" t="n">
         <v>46323</v>
       </c>
       <c r="D23" s="3" t="n">
@@ -12058,7 +12058,7 @@
           <t>GE</t>
         </is>
       </c>
-      <c r="C24" s="4" t="n">
+      <c r="C24" s="6" t="n">
         <v>46325</v>
       </c>
       <c r="D24" s="3" t="n">
@@ -12081,7 +12081,7 @@
           <t>GE</t>
         </is>
       </c>
-      <c r="C25" s="4" t="n">
+      <c r="C25" s="6" t="n">
         <v>46326</v>
       </c>
       <c r="D25" s="3" t="n">
@@ -12104,7 +12104,7 @@
           <t>GE</t>
         </is>
       </c>
-      <c r="C26" s="4" t="n">
+      <c r="C26" s="6" t="n">
         <v>46324</v>
       </c>
       <c r="D26" s="3" t="n">
@@ -12127,7 +12127,7 @@
           <t>GE</t>
         </is>
       </c>
-      <c r="C27" s="4" t="n">
+      <c r="C27" s="6" t="n">
         <v>46321</v>
       </c>
       <c r="D27" s="3" t="n">
@@ -12150,7 +12150,7 @@
           <t>GE</t>
         </is>
       </c>
-      <c r="C28" s="4" t="n">
+      <c r="C28" s="6" t="n">
         <v>46321</v>
       </c>
       <c r="D28" s="3" t="n">
@@ -12173,7 +12173,7 @@
           <t>GE</t>
         </is>
       </c>
-      <c r="C29" s="4" t="n">
+      <c r="C29" s="6" t="n">
         <v>46321</v>
       </c>
       <c r="D29" s="3" t="n">
@@ -12196,7 +12196,7 @@
           <t>GE</t>
         </is>
       </c>
-      <c r="C30" s="4" t="n">
+      <c r="C30" s="6" t="n">
         <v>46326</v>
       </c>
       <c r="D30" s="3" t="n">
@@ -12219,7 +12219,7 @@
           <t>GE</t>
         </is>
       </c>
-      <c r="C31" s="4" t="n">
+      <c r="C31" s="6" t="n">
         <v>46322</v>
       </c>
       <c r="D31" s="3" t="n">
@@ -12242,7 +12242,7 @@
           <t>GE</t>
         </is>
       </c>
-      <c r="C32" s="4" t="n">
+      <c r="C32" s="6" t="n">
         <v>46326</v>
       </c>
       <c r="D32" s="3" t="n">
@@ -12265,7 +12265,7 @@
           <t>GE</t>
         </is>
       </c>
-      <c r="C33" s="4" t="n">
+      <c r="C33" s="6" t="n">
         <v>46321</v>
       </c>
       <c r="D33" s="3" t="n">
@@ -12288,7 +12288,7 @@
           <t>GE</t>
         </is>
       </c>
-      <c r="C34" s="4" t="n">
+      <c r="C34" s="6" t="n">
         <v>46324</v>
       </c>
       <c r="D34" s="3" t="n">
@@ -12311,7 +12311,7 @@
           <t>GE</t>
         </is>
       </c>
-      <c r="C35" s="4" t="n">
+      <c r="C35" s="6" t="n">
         <v>46323</v>
       </c>
       <c r="D35" s="3" t="n">
@@ -12334,7 +12334,7 @@
           <t>GE</t>
         </is>
       </c>
-      <c r="C36" s="4" t="n">
+      <c r="C36" s="6" t="n">
         <v>46325</v>
       </c>
       <c r="D36" s="3" t="n">
@@ -12357,7 +12357,7 @@
           <t>GE</t>
         </is>
       </c>
-      <c r="C37" s="4" t="n">
+      <c r="C37" s="6" t="n">
         <v>46325</v>
       </c>
       <c r="D37" s="3" t="n">
@@ -12380,7 +12380,7 @@
           <t>GE</t>
         </is>
       </c>
-      <c r="C38" s="4" t="n">
+      <c r="C38" s="6" t="n">
         <v>46321</v>
       </c>
       <c r="D38" s="3" t="n">
@@ -12403,7 +12403,7 @@
           <t>GE</t>
         </is>
       </c>
-      <c r="C39" s="4" t="n">
+      <c r="C39" s="6" t="n">
         <v>46323</v>
       </c>
       <c r="D39" s="3" t="n">
@@ -12426,7 +12426,7 @@
           <t>GE</t>
         </is>
       </c>
-      <c r="C40" s="4" t="n">
+      <c r="C40" s="6" t="n">
         <v>46322</v>
       </c>
       <c r="D40" s="3" t="n">
@@ -12449,7 +12449,7 @@
           <t>GE</t>
         </is>
       </c>
-      <c r="C41" s="4" t="n">
+      <c r="C41" s="6" t="n">
         <v>46323</v>
       </c>
       <c r="D41" s="3" t="n">
@@ -12472,7 +12472,7 @@
           <t>GE</t>
         </is>
       </c>
-      <c r="C42" s="4" t="n">
+      <c r="C42" s="6" t="n">
         <v>46324</v>
       </c>
       <c r="D42" s="3" t="n">
@@ -12495,7 +12495,7 @@
           <t>GE</t>
         </is>
       </c>
-      <c r="C43" s="4" t="n">
+      <c r="C43" s="6" t="n">
         <v>46321</v>
       </c>
       <c r="D43" s="3" t="n">
@@ -12518,7 +12518,7 @@
           <t>GE</t>
         </is>
       </c>
-      <c r="C44" s="4" t="n">
+      <c r="C44" s="6" t="n">
         <v>46323</v>
       </c>
       <c r="D44" s="3" t="n">
@@ -12541,7 +12541,7 @@
           <t>GE</t>
         </is>
       </c>
-      <c r="C45" s="4" t="n">
+      <c r="C45" s="6" t="n">
         <v>46325</v>
       </c>
       <c r="D45" s="3" t="n">
@@ -12564,7 +12564,7 @@
           <t>GE</t>
         </is>
       </c>
-      <c r="C46" s="4" t="n">
+      <c r="C46" s="6" t="n">
         <v>46322</v>
       </c>
       <c r="D46" s="3" t="n">
@@ -12587,7 +12587,7 @@
           <t>GE</t>
         </is>
       </c>
-      <c r="C47" s="4" t="n">
+      <c r="C47" s="6" t="n">
         <v>46324</v>
       </c>
       <c r="D47" s="3" t="n">
@@ -12610,7 +12610,7 @@
           <t>GE</t>
         </is>
       </c>
-      <c r="C48" s="4" t="n">
+      <c r="C48" s="6" t="n">
         <v>46325</v>
       </c>
       <c r="D48" s="3" t="n">
@@ -12633,7 +12633,7 @@
           <t>GE</t>
         </is>
       </c>
-      <c r="C49" s="4" t="n">
+      <c r="C49" s="6" t="n">
         <v>46321</v>
       </c>
       <c r="D49" s="3" t="n">
@@ -12656,7 +12656,7 @@
           <t>GE</t>
         </is>
       </c>
-      <c r="C50" s="4" t="n">
+      <c r="C50" s="6" t="n">
         <v>46322</v>
       </c>
       <c r="D50" s="3" t="n">
@@ -12679,7 +12679,7 @@
           <t>GE</t>
         </is>
       </c>
-      <c r="C51" s="4" t="n">
+      <c r="C51" s="6" t="n">
         <v>46323</v>
       </c>
       <c r="D51" s="3" t="n">
@@ -12702,7 +12702,7 @@
           <t>GE</t>
         </is>
       </c>
-      <c r="C52" s="4" t="n">
+      <c r="C52" s="6" t="n">
         <v>46323</v>
       </c>
       <c r="D52" s="3" t="n">
@@ -12725,7 +12725,7 @@
           <t>GE</t>
         </is>
       </c>
-      <c r="C53" s="4" t="n">
+      <c r="C53" s="6" t="n">
         <v>46321</v>
       </c>
       <c r="D53" s="3" t="n">
@@ -12748,7 +12748,7 @@
           <t>GE</t>
         </is>
       </c>
-      <c r="C54" s="4" t="n">
+      <c r="C54" s="6" t="n">
         <v>46322</v>
       </c>
       <c r="D54" s="3" t="n">
@@ -12771,7 +12771,7 @@
           <t>GE</t>
         </is>
       </c>
-      <c r="C55" s="4" t="n">
+      <c r="C55" s="6" t="n">
         <v>46326</v>
       </c>
       <c r="D55" s="3" t="n">
@@ -12794,7 +12794,7 @@
           <t>GE</t>
         </is>
       </c>
-      <c r="C56" s="4" t="n">
+      <c r="C56" s="6" t="n">
         <v>46325</v>
       </c>
       <c r="D56" s="3" t="n">
@@ -12817,7 +12817,7 @@
           <t>GE</t>
         </is>
       </c>
-      <c r="C57" s="4" t="n">
+      <c r="C57" s="6" t="n">
         <v>46324</v>
       </c>
       <c r="D57" s="3" t="n">
@@ -12840,7 +12840,7 @@
           <t>GE</t>
         </is>
       </c>
-      <c r="C58" s="4" t="n">
+      <c r="C58" s="6" t="n">
         <v>46322</v>
       </c>
       <c r="D58" s="3" t="n">
@@ -12863,7 +12863,7 @@
           <t>GE</t>
         </is>
       </c>
-      <c r="C59" s="4" t="n">
+      <c r="C59" s="6" t="n">
         <v>46321</v>
       </c>
       <c r="D59" s="3" t="n">
@@ -12886,7 +12886,7 @@
           <t>GE</t>
         </is>
       </c>
-      <c r="C60" s="4" t="n">
+      <c r="C60" s="6" t="n">
         <v>46323</v>
       </c>
       <c r="D60" s="3" t="n">
@@ -12909,7 +12909,7 @@
           <t>GE</t>
         </is>
       </c>
-      <c r="C61" s="4" t="n">
+      <c r="C61" s="6" t="n">
         <v>46324</v>
       </c>
       <c r="D61" s="3" t="n">
@@ -12932,7 +12932,7 @@
           <t>GE</t>
         </is>
       </c>
-      <c r="C62" s="4" t="n">
+      <c r="C62" s="6" t="n">
         <v>46326</v>
       </c>
       <c r="D62" s="3" t="n">
@@ -12955,7 +12955,7 @@
           <t>GE</t>
         </is>
       </c>
-      <c r="C63" s="4" t="n">
+      <c r="C63" s="6" t="n">
         <v>46323</v>
       </c>
       <c r="D63" s="3" t="n">
@@ -12978,7 +12978,7 @@
           <t>GE</t>
         </is>
       </c>
-      <c r="C64" s="4" t="n">
+      <c r="C64" s="6" t="n">
         <v>46324</v>
       </c>
       <c r="D64" s="3" t="n">
@@ -13001,7 +13001,7 @@
           <t>GE</t>
         </is>
       </c>
-      <c r="C65" s="4" t="n">
+      <c r="C65" s="6" t="n">
         <v>46322</v>
       </c>
       <c r="D65" s="3" t="n">
@@ -13024,7 +13024,7 @@
           <t>GE</t>
         </is>
       </c>
-      <c r="C66" s="4" t="n">
+      <c r="C66" s="6" t="n">
         <v>46323</v>
       </c>
       <c r="D66" s="3" t="n">
@@ -13047,7 +13047,7 @@
           <t>GE</t>
         </is>
       </c>
-      <c r="C67" s="4" t="n">
+      <c r="C67" s="6" t="n">
         <v>46325</v>
       </c>
       <c r="D67" s="3" t="n">
@@ -13070,7 +13070,7 @@
           <t>GE</t>
         </is>
       </c>
-      <c r="C68" s="4" t="n">
+      <c r="C68" s="6" t="n">
         <v>46324</v>
       </c>
       <c r="D68" s="3" t="n">
@@ -13093,7 +13093,7 @@
           <t>GE</t>
         </is>
       </c>
-      <c r="C69" s="4" t="n">
+      <c r="C69" s="6" t="n">
         <v>46324</v>
       </c>
       <c r="D69" s="3" t="n">
@@ -13116,7 +13116,7 @@
           <t>GE</t>
         </is>
       </c>
-      <c r="C70" s="4" t="n">
+      <c r="C70" s="6" t="n">
         <v>46321</v>
       </c>
       <c r="D70" s="3" t="n">
@@ -13139,7 +13139,7 @@
           <t>GE</t>
         </is>
       </c>
-      <c r="C71" s="4" t="n">
+      <c r="C71" s="6" t="n">
         <v>46326</v>
       </c>
       <c r="D71" s="3" t="n">
@@ -13162,7 +13162,7 @@
           <t>GE</t>
         </is>
       </c>
-      <c r="C72" s="4" t="n">
+      <c r="C72" s="6" t="n">
         <v>46323</v>
       </c>
       <c r="D72" s="3" t="n">
@@ -13185,7 +13185,7 @@
           <t>GE</t>
         </is>
       </c>
-      <c r="C73" s="4" t="n">
+      <c r="C73" s="6" t="n">
         <v>46325</v>
       </c>
       <c r="D73" s="3" t="n">
@@ -13208,7 +13208,7 @@
           <t>GE</t>
         </is>
       </c>
-      <c r="C74" s="4" t="n">
+      <c r="C74" s="6" t="n">
         <v>46324</v>
       </c>
       <c r="D74" s="3" t="n">
@@ -13231,7 +13231,7 @@
           <t>GE</t>
         </is>
       </c>
-      <c r="C75" s="4" t="n">
+      <c r="C75" s="6" t="n">
         <v>46321</v>
       </c>
       <c r="D75" s="3" t="n">
@@ -13254,7 +13254,7 @@
           <t>GE</t>
         </is>
       </c>
-      <c r="C76" s="4" t="n">
+      <c r="C76" s="6" t="n">
         <v>46321</v>
       </c>
       <c r="D76" s="3" t="n">
@@ -13277,7 +13277,7 @@
           <t>GE</t>
         </is>
       </c>
-      <c r="C77" s="4" t="n">
+      <c r="C77" s="6" t="n">
         <v>46322</v>
       </c>
       <c r="D77" s="3" t="n">
@@ -13300,7 +13300,7 @@
           <t>GE</t>
         </is>
       </c>
-      <c r="C78" s="4" t="n">
+      <c r="C78" s="6" t="n">
         <v>46324</v>
       </c>
       <c r="D78" s="3" t="n">
@@ -13323,7 +13323,7 @@
           <t>GE</t>
         </is>
       </c>
-      <c r="C79" s="4" t="n">
+      <c r="C79" s="6" t="n">
         <v>46321</v>
       </c>
       <c r="D79" s="3" t="n">
@@ -13346,7 +13346,7 @@
           <t>GE</t>
         </is>
       </c>
-      <c r="C80" s="4" t="n">
+      <c r="C80" s="6" t="n">
         <v>46321</v>
       </c>
       <c r="D80" s="3" t="n">
@@ -13369,7 +13369,7 @@
           <t>GE</t>
         </is>
       </c>
-      <c r="C81" s="4" t="n">
+      <c r="C81" s="6" t="n">
         <v>46321</v>
       </c>
       <c r="D81" s="3" t="n">
@@ -13392,7 +13392,7 @@
           <t>GE</t>
         </is>
       </c>
-      <c r="C82" s="4" t="n">
+      <c r="C82" s="6" t="n">
         <v>46324</v>
       </c>
       <c r="D82" s="3" t="n">
@@ -13415,7 +13415,7 @@
           <t>GE</t>
         </is>
       </c>
-      <c r="C83" s="4" t="n">
+      <c r="C83" s="6" t="n">
         <v>46324</v>
       </c>
       <c r="D83" s="3" t="n">
@@ -13438,7 +13438,7 @@
           <t>GE</t>
         </is>
       </c>
-      <c r="C84" s="4" t="n">
+      <c r="C84" s="6" t="n">
         <v>46322</v>
       </c>
       <c r="D84" s="3" t="n">
@@ -13461,7 +13461,7 @@
           <t>GE</t>
         </is>
       </c>
-      <c r="C85" s="4" t="n">
+      <c r="C85" s="6" t="n">
         <v>46323</v>
       </c>
       <c r="D85" s="3" t="n">
@@ -13484,7 +13484,7 @@
           <t>GE</t>
         </is>
       </c>
-      <c r="C86" s="4" t="n">
+      <c r="C86" s="6" t="n">
         <v>46325</v>
       </c>
       <c r="D86" s="3" t="n">
@@ -13507,7 +13507,7 @@
           <t>GE</t>
         </is>
       </c>
-      <c r="C87" s="4" t="n">
+      <c r="C87" s="6" t="n">
         <v>46323</v>
       </c>
       <c r="D87" s="3" t="n">
@@ -13530,7 +13530,7 @@
           <t>GE</t>
         </is>
       </c>
-      <c r="C88" s="4" t="n">
+      <c r="C88" s="6" t="n">
         <v>46324</v>
       </c>
       <c r="D88" s="3" t="n">
@@ -13553,7 +13553,7 @@
           <t>GE</t>
         </is>
       </c>
-      <c r="C89" s="4" t="n">
+      <c r="C89" s="6" t="n">
         <v>46324</v>
       </c>
       <c r="D89" s="3" t="n">
@@ -13576,7 +13576,7 @@
           <t>GE</t>
         </is>
       </c>
-      <c r="C90" s="4" t="n">
+      <c r="C90" s="6" t="n">
         <v>46324</v>
       </c>
       <c r="D90" s="3" t="n">
@@ -13599,7 +13599,7 @@
           <t>GE</t>
         </is>
       </c>
-      <c r="C91" s="4" t="n">
+      <c r="C91" s="6" t="n">
         <v>46326</v>
       </c>
       <c r="D91" s="3" t="n">
@@ -13622,7 +13622,7 @@
           <t>GE</t>
         </is>
       </c>
-      <c r="C92" s="4" t="n">
+      <c r="C92" s="6" t="n">
         <v>46326</v>
       </c>
       <c r="D92" s="3" t="n">
@@ -13645,7 +13645,7 @@
           <t>GE</t>
         </is>
       </c>
-      <c r="C93" s="4" t="n">
+      <c r="C93" s="6" t="n">
         <v>46324</v>
       </c>
       <c r="D93" s="3" t="n">
@@ -13668,7 +13668,7 @@
           <t>GE</t>
         </is>
       </c>
-      <c r="C94" s="4" t="n">
+      <c r="C94" s="6" t="n">
         <v>46326</v>
       </c>
       <c r="D94" s="3" t="n">
@@ -13691,7 +13691,7 @@
           <t>GE</t>
         </is>
       </c>
-      <c r="C95" s="4" t="n">
+      <c r="C95" s="6" t="n">
         <v>46324</v>
       </c>
       <c r="D95" s="3" t="n">
@@ -13714,7 +13714,7 @@
           <t>GE</t>
         </is>
       </c>
-      <c r="C96" s="4" t="n">
+      <c r="C96" s="6" t="n">
         <v>46326</v>
       </c>
       <c r="D96" s="3" t="n">
@@ -13737,7 +13737,7 @@
           <t>GE</t>
         </is>
       </c>
-      <c r="C97" s="4" t="n">
+      <c r="C97" s="6" t="n">
         <v>46326</v>
       </c>
       <c r="D97" s="3" t="n">
@@ -13760,7 +13760,7 @@
           <t>GE</t>
         </is>
       </c>
-      <c r="C98" s="4" t="n">
+      <c r="C98" s="6" t="n">
         <v>46321</v>
       </c>
       <c r="D98" s="3" t="n">
@@ -13783,7 +13783,7 @@
           <t>GE</t>
         </is>
       </c>
-      <c r="C99" s="4" t="n">
+      <c r="C99" s="6" t="n">
         <v>46326</v>
       </c>
       <c r="D99" s="3" t="n">
@@ -13806,7 +13806,7 @@
           <t>GE</t>
         </is>
       </c>
-      <c r="C100" s="4" t="n">
+      <c r="C100" s="6" t="n">
         <v>46325</v>
       </c>
       <c r="D100" s="3" t="n">
@@ -13829,7 +13829,7 @@
           <t>GE</t>
         </is>
       </c>
-      <c r="C101" s="4" t="n">
+      <c r="C101" s="6" t="n">
         <v>46321</v>
       </c>
       <c r="D101" s="3" t="n">
@@ -13852,7 +13852,7 @@
           <t>GE</t>
         </is>
       </c>
-      <c r="C102" s="4" t="n">
+      <c r="C102" s="6" t="n">
         <v>46323</v>
       </c>
       <c r="D102" s="3" t="n">
@@ -13875,7 +13875,7 @@
           <t>GE</t>
         </is>
       </c>
-      <c r="C103" s="4" t="n">
+      <c r="C103" s="6" t="n">
         <v>46322</v>
       </c>
       <c r="D103" s="3" t="n">
@@ -13898,7 +13898,7 @@
           <t>GE</t>
         </is>
       </c>
-      <c r="C104" s="4" t="n">
+      <c r="C104" s="6" t="n">
         <v>46323</v>
       </c>
       <c r="D104" s="3" t="n">
@@ -13921,7 +13921,7 @@
           <t>GE</t>
         </is>
       </c>
-      <c r="C105" s="4" t="n">
+      <c r="C105" s="6" t="n">
         <v>46325</v>
       </c>
       <c r="D105" s="3" t="n">
@@ -13944,7 +13944,7 @@
           <t>GE</t>
         </is>
       </c>
-      <c r="C106" s="4" t="n">
+      <c r="C106" s="6" t="n">
         <v>46324</v>
       </c>
       <c r="D106" s="3" t="n">
@@ -13967,7 +13967,7 @@
           <t>GE</t>
         </is>
       </c>
-      <c r="C107" s="4" t="n">
+      <c r="C107" s="6" t="n">
         <v>46322</v>
       </c>
       <c r="D107" s="3" t="n">
@@ -13990,7 +13990,7 @@
           <t>GE</t>
         </is>
       </c>
-      <c r="C108" s="4" t="n">
+      <c r="C108" s="6" t="n">
         <v>46324</v>
       </c>
       <c r="D108" s="3" t="n">
@@ -14013,7 +14013,7 @@
           <t>GE</t>
         </is>
       </c>
-      <c r="C109" s="4" t="n">
+      <c r="C109" s="6" t="n">
         <v>46323</v>
       </c>
       <c r="D109" s="3" t="n">
@@ -31139,7 +31139,7 @@
           <t>Participación completa en el cuaderno simulado</t>
         </is>
       </c>
-      <c r="E5" s="4" t="n">
+      <c r="E5" s="6" t="n">
         <v>46322</v>
       </c>
       <c r="F5" s="3" t="inlineStr">
@@ -31167,7 +31167,7 @@
           <t>Participación completa en el cuaderno simulado</t>
         </is>
       </c>
-      <c r="E6" s="4" t="n">
+      <c r="E6" s="6" t="n">
         <v>46321</v>
       </c>
       <c r="F6" s="3" t="inlineStr">
@@ -31195,7 +31195,7 @@
           <t>Participación completa en el cuaderno simulado</t>
         </is>
       </c>
-      <c r="E7" s="4" t="n">
+      <c r="E7" s="6" t="n">
         <v>46321</v>
       </c>
       <c r="F7" s="3" t="inlineStr">
@@ -31223,7 +31223,7 @@
           <t>Participación completa en el cuaderno simulado</t>
         </is>
       </c>
-      <c r="E8" s="4" t="n">
+      <c r="E8" s="6" t="n">
         <v>46324</v>
       </c>
       <c r="F8" s="3" t="inlineStr">
@@ -31251,7 +31251,7 @@
           <t>Participación completa en el cuaderno simulado</t>
         </is>
       </c>
-      <c r="E9" s="4" t="n">
+      <c r="E9" s="6" t="n">
         <v>46321</v>
       </c>
       <c r="F9" s="3" t="inlineStr">
@@ -31279,7 +31279,7 @@
           <t>Participación completa en el cuaderno simulado</t>
         </is>
       </c>
-      <c r="E10" s="4" t="n">
+      <c r="E10" s="6" t="n">
         <v>46322</v>
       </c>
       <c r="F10" s="3" t="inlineStr">
@@ -31307,7 +31307,7 @@
           <t>Participación completa en el cuaderno simulado</t>
         </is>
       </c>
-      <c r="E11" s="4" t="n">
+      <c r="E11" s="6" t="n">
         <v>46324</v>
       </c>
       <c r="F11" s="3" t="inlineStr">
@@ -31335,7 +31335,7 @@
           <t>Participación completa en el cuaderno simulado</t>
         </is>
       </c>
-      <c r="E12" s="4" t="n">
+      <c r="E12" s="6" t="n">
         <v>46321</v>
       </c>
       <c r="F12" s="3" t="inlineStr">
@@ -31363,7 +31363,7 @@
           <t>Participación completa en el cuaderno simulado</t>
         </is>
       </c>
-      <c r="E13" s="4" t="n">
+      <c r="E13" s="6" t="n">
         <v>46322</v>
       </c>
       <c r="F13" s="3" t="inlineStr">
@@ -31391,7 +31391,7 @@
           <t>Participación completa en el cuaderno simulado</t>
         </is>
       </c>
-      <c r="E14" s="4" t="n">
+      <c r="E14" s="6" t="n">
         <v>46322</v>
       </c>
       <c r="F14" s="3" t="inlineStr">
@@ -31419,7 +31419,7 @@
           <t>Participación completa en el cuaderno simulado</t>
         </is>
       </c>
-      <c r="E15" s="4" t="n">
+      <c r="E15" s="6" t="n">
         <v>46321</v>
       </c>
       <c r="F15" s="3" t="inlineStr">
@@ -31447,7 +31447,7 @@
           <t>Retiro sin postest: no completó las sesiones mínimas</t>
         </is>
       </c>
-      <c r="E16" s="4" t="n">
+      <c r="E16" s="6" t="n">
         <v>46316</v>
       </c>
       <c r="F16" s="3" t="inlineStr">
@@ -31475,7 +31475,7 @@
           <t>Participación completa en el cuaderno simulado</t>
         </is>
       </c>
-      <c r="E17" s="4" t="n">
+      <c r="E17" s="6" t="n">
         <v>46322</v>
       </c>
       <c r="F17" s="3" t="inlineStr">
@@ -31503,7 +31503,7 @@
           <t>Participación completa en el cuaderno simulado</t>
         </is>
       </c>
-      <c r="E18" s="4" t="n">
+      <c r="E18" s="6" t="n">
         <v>46322</v>
       </c>
       <c r="F18" s="3" t="inlineStr">
@@ -31531,7 +31531,7 @@
           <t>Participación completa en el cuaderno simulado</t>
         </is>
       </c>
-      <c r="E19" s="4" t="n">
+      <c r="E19" s="6" t="n">
         <v>46321</v>
       </c>
       <c r="F19" s="3" t="inlineStr">
@@ -31559,7 +31559,7 @@
           <t>Participación completa en el cuaderno simulado</t>
         </is>
       </c>
-      <c r="E20" s="4" t="n">
+      <c r="E20" s="6" t="n">
         <v>46323</v>
       </c>
       <c r="F20" s="3" t="inlineStr">
@@ -31587,7 +31587,7 @@
           <t>Participación completa en el cuaderno simulado</t>
         </is>
       </c>
-      <c r="E21" s="4" t="n">
+      <c r="E21" s="6" t="n">
         <v>46321</v>
       </c>
       <c r="F21" s="3" t="inlineStr">
@@ -31615,7 +31615,7 @@
           <t>Participación completa en el cuaderno simulado</t>
         </is>
       </c>
-      <c r="E22" s="4" t="n">
+      <c r="E22" s="6" t="n">
         <v>46323</v>
       </c>
       <c r="F22" s="3" t="inlineStr">
@@ -31643,7 +31643,7 @@
           <t>Participación completa en el cuaderno simulado</t>
         </is>
       </c>
-      <c r="E23" s="4" t="n">
+      <c r="E23" s="6" t="n">
         <v>46325</v>
       </c>
       <c r="F23" s="3" t="inlineStr">
@@ -31671,7 +31671,7 @@
           <t>Participación completa en el cuaderno simulado</t>
         </is>
       </c>
-      <c r="E24" s="4" t="n">
+      <c r="E24" s="6" t="n">
         <v>46323</v>
       </c>
       <c r="F24" s="3" t="inlineStr">
@@ -31699,7 +31699,7 @@
           <t>Participación completa en el cuaderno simulado</t>
         </is>
       </c>
-      <c r="E25" s="4" t="n">
+      <c r="E25" s="6" t="n">
         <v>46325</v>
       </c>
       <c r="F25" s="3" t="inlineStr">
@@ -31727,7 +31727,7 @@
           <t>Participación completa en el cuaderno simulado</t>
         </is>
       </c>
-      <c r="E26" s="4" t="n">
+      <c r="E26" s="6" t="n">
         <v>46326</v>
       </c>
       <c r="F26" s="3" t="inlineStr">
@@ -31755,7 +31755,7 @@
           <t>Participación completa en el cuaderno simulado</t>
         </is>
       </c>
-      <c r="E27" s="4" t="n">
+      <c r="E27" s="6" t="n">
         <v>46324</v>
       </c>
       <c r="F27" s="3" t="inlineStr">
@@ -31783,7 +31783,7 @@
           <t>Participación completa en el cuaderno simulado</t>
         </is>
       </c>
-      <c r="E28" s="4" t="n">
+      <c r="E28" s="6" t="n">
         <v>46321</v>
       </c>
       <c r="F28" s="3" t="inlineStr">
@@ -31811,7 +31811,7 @@
           <t>Participación completa en el cuaderno simulado</t>
         </is>
       </c>
-      <c r="E29" s="4" t="n">
+      <c r="E29" s="6" t="n">
         <v>46321</v>
       </c>
       <c r="F29" s="3" t="inlineStr">
@@ -31839,7 +31839,7 @@
           <t>Participación completa en el cuaderno simulado</t>
         </is>
       </c>
-      <c r="E30" s="4" t="n">
+      <c r="E30" s="6" t="n">
         <v>46321</v>
       </c>
       <c r="F30" s="3" t="inlineStr">
@@ -31867,7 +31867,7 @@
           <t>Participación completa en el cuaderno simulado</t>
         </is>
       </c>
-      <c r="E31" s="4" t="n">
+      <c r="E31" s="6" t="n">
         <v>46326</v>
       </c>
       <c r="F31" s="3" t="inlineStr">
@@ -31895,7 +31895,7 @@
           <t>Retiro sin postest: no completó las sesiones mínimas</t>
         </is>
       </c>
-      <c r="E32" s="4" t="n">
+      <c r="E32" s="6" t="n">
         <v>46316</v>
       </c>
       <c r="F32" s="3" t="inlineStr">
@@ -31923,7 +31923,7 @@
           <t>Participación completa en el cuaderno simulado</t>
         </is>
       </c>
-      <c r="E33" s="4" t="n">
+      <c r="E33" s="6" t="n">
         <v>46322</v>
       </c>
       <c r="F33" s="3" t="inlineStr">
@@ -31951,7 +31951,7 @@
           <t>Participación completa en el cuaderno simulado</t>
         </is>
       </c>
-      <c r="E34" s="4" t="n">
+      <c r="E34" s="6" t="n">
         <v>46326</v>
       </c>
       <c r="F34" s="3" t="inlineStr">
@@ -31979,7 +31979,7 @@
           <t>Participación completa en el cuaderno simulado</t>
         </is>
       </c>
-      <c r="E35" s="4" t="n">
+      <c r="E35" s="6" t="n">
         <v>46321</v>
       </c>
       <c r="F35" s="3" t="inlineStr">
@@ -32007,7 +32007,7 @@
           <t>Participación completa en el cuaderno simulado</t>
         </is>
       </c>
-      <c r="E36" s="4" t="n">
+      <c r="E36" s="6" t="n">
         <v>46324</v>
       </c>
       <c r="F36" s="3" t="inlineStr">
@@ -32035,7 +32035,7 @@
           <t>Participación completa en el cuaderno simulado</t>
         </is>
       </c>
-      <c r="E37" s="4" t="n">
+      <c r="E37" s="6" t="n">
         <v>46323</v>
       </c>
       <c r="F37" s="3" t="inlineStr">
@@ -32063,7 +32063,7 @@
           <t>Participación completa en el cuaderno simulado</t>
         </is>
       </c>
-      <c r="E38" s="4" t="n">
+      <c r="E38" s="6" t="n">
         <v>46325</v>
       </c>
       <c r="F38" s="3" t="inlineStr">
@@ -32091,7 +32091,7 @@
           <t>Participación completa en el cuaderno simulado</t>
         </is>
       </c>
-      <c r="E39" s="4" t="n">
+      <c r="E39" s="6" t="n">
         <v>46325</v>
       </c>
       <c r="F39" s="3" t="inlineStr">
@@ -32119,7 +32119,7 @@
           <t>Participación completa en el cuaderno simulado</t>
         </is>
       </c>
-      <c r="E40" s="4" t="n">
+      <c r="E40" s="6" t="n">
         <v>46321</v>
       </c>
       <c r="F40" s="3" t="inlineStr">
@@ -32147,7 +32147,7 @@
           <t>Participación completa en el cuaderno simulado</t>
         </is>
       </c>
-      <c r="E41" s="4" t="n">
+      <c r="E41" s="6" t="n">
         <v>46323</v>
       </c>
       <c r="F41" s="3" t="inlineStr">
@@ -32175,7 +32175,7 @@
           <t>Participación completa en el cuaderno simulado</t>
         </is>
       </c>
-      <c r="E42" s="4" t="n">
+      <c r="E42" s="6" t="n">
         <v>46322</v>
       </c>
       <c r="F42" s="3" t="inlineStr">
@@ -32203,7 +32203,7 @@
           <t>Participación completa en el cuaderno simulado</t>
         </is>
       </c>
-      <c r="E43" s="4" t="n">
+      <c r="E43" s="6" t="n">
         <v>46323</v>
       </c>
       <c r="F43" s="3" t="inlineStr">
@@ -32231,7 +32231,7 @@
           <t>Participación completa en el cuaderno simulado</t>
         </is>
       </c>
-      <c r="E44" s="4" t="n">
+      <c r="E44" s="6" t="n">
         <v>46324</v>
       </c>
       <c r="F44" s="3" t="inlineStr">
@@ -32259,7 +32259,7 @@
           <t>Participación completa en el cuaderno simulado</t>
         </is>
       </c>
-      <c r="E45" s="4" t="n">
+      <c r="E45" s="6" t="n">
         <v>46321</v>
       </c>
       <c r="F45" s="3" t="inlineStr">
@@ -32287,7 +32287,7 @@
           <t>Participación completa en el cuaderno simulado</t>
         </is>
       </c>
-      <c r="E46" s="4" t="n">
+      <c r="E46" s="6" t="n">
         <v>46323</v>
       </c>
       <c r="F46" s="3" t="inlineStr">
@@ -32315,7 +32315,7 @@
           <t>Participación completa en el cuaderno simulado</t>
         </is>
       </c>
-      <c r="E47" s="4" t="n">
+      <c r="E47" s="6" t="n">
         <v>46325</v>
       </c>
       <c r="F47" s="3" t="inlineStr">
@@ -32343,7 +32343,7 @@
           <t>Participación completa en el cuaderno simulado</t>
         </is>
       </c>
-      <c r="E48" s="4" t="n">
+      <c r="E48" s="6" t="n">
         <v>46322</v>
       </c>
       <c r="F48" s="3" t="inlineStr">
@@ -32371,7 +32371,7 @@
           <t>Retiro sin postest: no completó las sesiones mínimas</t>
         </is>
       </c>
-      <c r="E49" s="4" t="n">
+      <c r="E49" s="6" t="n">
         <v>46316</v>
       </c>
       <c r="F49" s="3" t="inlineStr">
@@ -32399,7 +32399,7 @@
           <t>Participación completa en el cuaderno simulado</t>
         </is>
       </c>
-      <c r="E50" s="4" t="n">
+      <c r="E50" s="6" t="n">
         <v>46324</v>
       </c>
       <c r="F50" s="3" t="inlineStr">
@@ -32427,7 +32427,7 @@
           <t>Participación completa en el cuaderno simulado</t>
         </is>
       </c>
-      <c r="E51" s="4" t="n">
+      <c r="E51" s="6" t="n">
         <v>46325</v>
       </c>
       <c r="F51" s="3" t="inlineStr">
@@ -32455,7 +32455,7 @@
           <t>Participación completa en el cuaderno simulado</t>
         </is>
       </c>
-      <c r="E52" s="4" t="n">
+      <c r="E52" s="6" t="n">
         <v>46321</v>
       </c>
       <c r="F52" s="3" t="inlineStr">
@@ -32483,7 +32483,7 @@
           <t>Participación completa en el cuaderno simulado</t>
         </is>
       </c>
-      <c r="E53" s="4" t="n">
+      <c r="E53" s="6" t="n">
         <v>46322</v>
       </c>
       <c r="F53" s="3" t="inlineStr">
@@ -32511,7 +32511,7 @@
           <t>Participación completa en el cuaderno simulado</t>
         </is>
       </c>
-      <c r="E54" s="4" t="n">
+      <c r="E54" s="6" t="n">
         <v>46323</v>
       </c>
       <c r="F54" s="3" t="inlineStr">
@@ -32539,7 +32539,7 @@
           <t>Participación completa en el cuaderno simulado</t>
         </is>
       </c>
-      <c r="E55" s="4" t="n">
+      <c r="E55" s="6" t="n">
         <v>46323</v>
       </c>
       <c r="F55" s="3" t="inlineStr">
@@ -32567,7 +32567,7 @@
           <t>Participación completa en el cuaderno simulado</t>
         </is>
       </c>
-      <c r="E56" s="4" t="n">
+      <c r="E56" s="6" t="n">
         <v>46321</v>
       </c>
       <c r="F56" s="3" t="inlineStr">
@@ -32595,7 +32595,7 @@
           <t>Participación completa en el cuaderno simulado</t>
         </is>
       </c>
-      <c r="E57" s="4" t="n">
+      <c r="E57" s="6" t="n">
         <v>46322</v>
       </c>
       <c r="F57" s="3" t="inlineStr">
@@ -32623,7 +32623,7 @@
           <t>Participación completa en el cuaderno simulado</t>
         </is>
       </c>
-      <c r="E58" s="4" t="n">
+      <c r="E58" s="6" t="n">
         <v>46326</v>
       </c>
       <c r="F58" s="3" t="inlineStr">
@@ -32651,7 +32651,7 @@
           <t>Participación completa en el cuaderno simulado</t>
         </is>
       </c>
-      <c r="E59" s="4" t="n">
+      <c r="E59" s="6" t="n">
         <v>46325</v>
       </c>
       <c r="F59" s="3" t="inlineStr">
@@ -32679,7 +32679,7 @@
           <t>Participación completa en el cuaderno simulado</t>
         </is>
       </c>
-      <c r="E60" s="4" t="n">
+      <c r="E60" s="6" t="n">
         <v>46324</v>
       </c>
       <c r="F60" s="3" t="inlineStr">
@@ -32707,7 +32707,7 @@
           <t>Participación completa en el cuaderno simulado</t>
         </is>
       </c>
-      <c r="E61" s="4" t="n">
+      <c r="E61" s="6" t="n">
         <v>46322</v>
       </c>
       <c r="F61" s="3" t="inlineStr">
@@ -32735,7 +32735,7 @@
           <t>Participación completa en el cuaderno simulado</t>
         </is>
       </c>
-      <c r="E62" s="4" t="n">
+      <c r="E62" s="6" t="n">
         <v>46321</v>
       </c>
       <c r="F62" s="3" t="inlineStr">
@@ -32763,7 +32763,7 @@
           <t>Participación completa en el cuaderno simulado</t>
         </is>
       </c>
-      <c r="E63" s="4" t="n">
+      <c r="E63" s="6" t="n">
         <v>46323</v>
       </c>
       <c r="F63" s="3" t="inlineStr">
@@ -32791,7 +32791,7 @@
           <t>Participación completa en el cuaderno simulado</t>
         </is>
       </c>
-      <c r="E64" s="4" t="n">
+      <c r="E64" s="6" t="n">
         <v>46324</v>
       </c>
       <c r="F64" s="3" t="inlineStr">
@@ -32819,7 +32819,7 @@
           <t>Participación completa en el cuaderno simulado</t>
         </is>
       </c>
-      <c r="E65" s="4" t="n">
+      <c r="E65" s="6" t="n">
         <v>46326</v>
       </c>
       <c r="F65" s="3" t="inlineStr">
@@ -32847,7 +32847,7 @@
           <t>Participación completa en el cuaderno simulado</t>
         </is>
       </c>
-      <c r="E66" s="4" t="n">
+      <c r="E66" s="6" t="n">
         <v>46323</v>
       </c>
       <c r="F66" s="3" t="inlineStr">
@@ -32875,7 +32875,7 @@
           <t>Participación completa en el cuaderno simulado</t>
         </is>
       </c>
-      <c r="E67" s="4" t="n">
+      <c r="E67" s="6" t="n">
         <v>46324</v>
       </c>
       <c r="F67" s="3" t="inlineStr">
@@ -32903,7 +32903,7 @@
           <t>Participación completa en el cuaderno simulado</t>
         </is>
       </c>
-      <c r="E68" s="4" t="n">
+      <c r="E68" s="6" t="n">
         <v>46322</v>
       </c>
       <c r="F68" s="3" t="inlineStr">
@@ -32931,7 +32931,7 @@
           <t>Participación completa en el cuaderno simulado</t>
         </is>
       </c>
-      <c r="E69" s="4" t="n">
+      <c r="E69" s="6" t="n">
         <v>46323</v>
       </c>
       <c r="F69" s="3" t="inlineStr">
@@ -32959,7 +32959,7 @@
           <t>Participación completa en el cuaderno simulado</t>
         </is>
       </c>
-      <c r="E70" s="4" t="n">
+      <c r="E70" s="6" t="n">
         <v>46325</v>
       </c>
       <c r="F70" s="3" t="inlineStr">
@@ -32987,7 +32987,7 @@
           <t>Participación completa en el cuaderno simulado</t>
         </is>
       </c>
-      <c r="E71" s="4" t="n">
+      <c r="E71" s="6" t="n">
         <v>46324</v>
       </c>
       <c r="F71" s="3" t="inlineStr">
@@ -33015,7 +33015,7 @@
           <t>Participación completa en el cuaderno simulado</t>
         </is>
       </c>
-      <c r="E72" s="4" t="n">
+      <c r="E72" s="6" t="n">
         <v>46324</v>
       </c>
       <c r="F72" s="3" t="inlineStr">
@@ -33043,7 +33043,7 @@
           <t>Participación completa en el cuaderno simulado</t>
         </is>
       </c>
-      <c r="E73" s="4" t="n">
+      <c r="E73" s="6" t="n">
         <v>46321</v>
       </c>
       <c r="F73" s="3" t="inlineStr">
@@ -33071,7 +33071,7 @@
           <t>Participación completa en el cuaderno simulado</t>
         </is>
       </c>
-      <c r="E74" s="4" t="n">
+      <c r="E74" s="6" t="n">
         <v>46326</v>
       </c>
       <c r="F74" s="3" t="inlineStr">
@@ -33099,7 +33099,7 @@
           <t>Participación completa en el cuaderno simulado</t>
         </is>
       </c>
-      <c r="E75" s="4" t="n">
+      <c r="E75" s="6" t="n">
         <v>46323</v>
       </c>
       <c r="F75" s="3" t="inlineStr">
@@ -33127,7 +33127,7 @@
           <t>Participación completa en el cuaderno simulado</t>
         </is>
       </c>
-      <c r="E76" s="4" t="n">
+      <c r="E76" s="6" t="n">
         <v>46325</v>
       </c>
       <c r="F76" s="3" t="inlineStr">
@@ -33155,7 +33155,7 @@
           <t>Participación completa en el cuaderno simulado</t>
         </is>
       </c>
-      <c r="E77" s="4" t="n">
+      <c r="E77" s="6" t="n">
         <v>46324</v>
       </c>
       <c r="F77" s="3" t="inlineStr">
@@ -33183,7 +33183,7 @@
           <t>Participación completa en el cuaderno simulado</t>
         </is>
       </c>
-      <c r="E78" s="4" t="n">
+      <c r="E78" s="6" t="n">
         <v>46321</v>
       </c>
       <c r="F78" s="3" t="inlineStr">
@@ -33211,7 +33211,7 @@
           <t>Participación completa en el cuaderno simulado</t>
         </is>
       </c>
-      <c r="E79" s="4" t="n">
+      <c r="E79" s="6" t="n">
         <v>46321</v>
       </c>
       <c r="F79" s="3" t="inlineStr">
@@ -33239,7 +33239,7 @@
           <t>Participación completa en el cuaderno simulado</t>
         </is>
       </c>
-      <c r="E80" s="4" t="n">
+      <c r="E80" s="6" t="n">
         <v>46322</v>
       </c>
       <c r="F80" s="3" t="inlineStr">
@@ -33267,7 +33267,7 @@
           <t>Participación completa en el cuaderno simulado</t>
         </is>
       </c>
-      <c r="E81" s="4" t="n">
+      <c r="E81" s="6" t="n">
         <v>46324</v>
       </c>
       <c r="F81" s="3" t="inlineStr">
@@ -33295,7 +33295,7 @@
           <t>Participación completa en el cuaderno simulado</t>
         </is>
       </c>
-      <c r="E82" s="4" t="n">
+      <c r="E82" s="6" t="n">
         <v>46321</v>
       </c>
       <c r="F82" s="3" t="inlineStr">
@@ -33323,7 +33323,7 @@
           <t>Participación completa en el cuaderno simulado</t>
         </is>
       </c>
-      <c r="E83" s="4" t="n">
+      <c r="E83" s="6" t="n">
         <v>46321</v>
       </c>
       <c r="F83" s="3" t="inlineStr">
@@ -33351,7 +33351,7 @@
           <t>Participación completa en el cuaderno simulado</t>
         </is>
       </c>
-      <c r="E84" s="4" t="n">
+      <c r="E84" s="6" t="n">
         <v>46321</v>
       </c>
       <c r="F84" s="3" t="inlineStr">
@@ -33379,7 +33379,7 @@
           <t>Participación completa en el cuaderno simulado</t>
         </is>
       </c>
-      <c r="E85" s="4" t="n">
+      <c r="E85" s="6" t="n">
         <v>46324</v>
       </c>
       <c r="F85" s="3" t="inlineStr">
@@ -33407,7 +33407,7 @@
           <t>Participación completa en el cuaderno simulado</t>
         </is>
       </c>
-      <c r="E86" s="4" t="n">
+      <c r="E86" s="6" t="n">
         <v>46324</v>
       </c>
       <c r="F86" s="3" t="inlineStr">
@@ -33435,7 +33435,7 @@
           <t>Participación completa en el cuaderno simulado</t>
         </is>
       </c>
-      <c r="E87" s="4" t="n">
+      <c r="E87" s="6" t="n">
         <v>46322</v>
       </c>
       <c r="F87" s="3" t="inlineStr">
@@ -33463,7 +33463,7 @@
           <t>Participación completa en el cuaderno simulado</t>
         </is>
       </c>
-      <c r="E88" s="4" t="n">
+      <c r="E88" s="6" t="n">
         <v>46323</v>
       </c>
       <c r="F88" s="3" t="inlineStr">
@@ -33491,7 +33491,7 @@
           <t>Participación completa en el cuaderno simulado</t>
         </is>
       </c>
-      <c r="E89" s="4" t="n">
+      <c r="E89" s="6" t="n">
         <v>46325</v>
       </c>
       <c r="F89" s="3" t="inlineStr">
@@ -33519,7 +33519,7 @@
           <t>Participación completa en el cuaderno simulado</t>
         </is>
       </c>
-      <c r="E90" s="4" t="n">
+      <c r="E90" s="6" t="n">
         <v>46323</v>
       </c>
       <c r="F90" s="3" t="inlineStr">
@@ -33547,7 +33547,7 @@
           <t>Participación completa en el cuaderno simulado</t>
         </is>
       </c>
-      <c r="E91" s="4" t="n">
+      <c r="E91" s="6" t="n">
         <v>46324</v>
       </c>
       <c r="F91" s="3" t="inlineStr">
@@ -33575,7 +33575,7 @@
           <t>Participación completa en el cuaderno simulado</t>
         </is>
       </c>
-      <c r="E92" s="4" t="n">
+      <c r="E92" s="6" t="n">
         <v>46324</v>
       </c>
       <c r="F92" s="3" t="inlineStr">
@@ -33603,7 +33603,7 @@
           <t>Participación completa en el cuaderno simulado</t>
         </is>
       </c>
-      <c r="E93" s="4" t="n">
+      <c r="E93" s="6" t="n">
         <v>46324</v>
       </c>
       <c r="F93" s="3" t="inlineStr">
@@ -33631,7 +33631,7 @@
           <t>Participación completa en el cuaderno simulado</t>
         </is>
       </c>
-      <c r="E94" s="4" t="n">
+      <c r="E94" s="6" t="n">
         <v>46326</v>
       </c>
       <c r="F94" s="3" t="inlineStr">
@@ -33659,7 +33659,7 @@
           <t>Participación completa en el cuaderno simulado</t>
         </is>
       </c>
-      <c r="E95" s="4" t="n">
+      <c r="E95" s="6" t="n">
         <v>46326</v>
       </c>
       <c r="F95" s="3" t="inlineStr">
@@ -33687,7 +33687,7 @@
           <t>Participación completa en el cuaderno simulado</t>
         </is>
       </c>
-      <c r="E96" s="4" t="n">
+      <c r="E96" s="6" t="n">
         <v>46324</v>
       </c>
       <c r="F96" s="3" t="inlineStr">
@@ -33715,7 +33715,7 @@
           <t>Participación completa en el cuaderno simulado</t>
         </is>
       </c>
-      <c r="E97" s="4" t="n">
+      <c r="E97" s="6" t="n">
         <v>46326</v>
       </c>
       <c r="F97" s="3" t="inlineStr">
@@ -33743,7 +33743,7 @@
           <t>Participación completa en el cuaderno simulado</t>
         </is>
       </c>
-      <c r="E98" s="4" t="n">
+      <c r="E98" s="6" t="n">
         <v>46324</v>
       </c>
       <c r="F98" s="3" t="inlineStr">
@@ -33771,7 +33771,7 @@
           <t>Participación completa en el cuaderno simulado</t>
         </is>
       </c>
-      <c r="E99" s="4" t="n">
+      <c r="E99" s="6" t="n">
         <v>46326</v>
       </c>
       <c r="F99" s="3" t="inlineStr">
@@ -33799,7 +33799,7 @@
           <t>Participación completa en el cuaderno simulado</t>
         </is>
       </c>
-      <c r="E100" s="4" t="n">
+      <c r="E100" s="6" t="n">
         <v>46326</v>
       </c>
       <c r="F100" s="3" t="inlineStr">
@@ -33827,7 +33827,7 @@
           <t>Participación completa en el cuaderno simulado</t>
         </is>
       </c>
-      <c r="E101" s="4" t="n">
+      <c r="E101" s="6" t="n">
         <v>46321</v>
       </c>
       <c r="F101" s="3" t="inlineStr">
@@ -33855,7 +33855,7 @@
           <t>Participación completa en el cuaderno simulado</t>
         </is>
       </c>
-      <c r="E102" s="4" t="n">
+      <c r="E102" s="6" t="n">
         <v>46326</v>
       </c>
       <c r="F102" s="3" t="inlineStr">
@@ -33883,7 +33883,7 @@
           <t>Participación completa en el cuaderno simulado</t>
         </is>
       </c>
-      <c r="E103" s="4" t="n">
+      <c r="E103" s="6" t="n">
         <v>46325</v>
       </c>
       <c r="F103" s="3" t="inlineStr">
@@ -33911,7 +33911,7 @@
           <t>Participación completa en el cuaderno simulado</t>
         </is>
       </c>
-      <c r="E104" s="4" t="n">
+      <c r="E104" s="6" t="n">
         <v>46321</v>
       </c>
       <c r="F104" s="3" t="inlineStr">
@@ -33939,7 +33939,7 @@
           <t>Participación completa en el cuaderno simulado</t>
         </is>
       </c>
-      <c r="E105" s="4" t="n">
+      <c r="E105" s="6" t="n">
         <v>46323</v>
       </c>
       <c r="F105" s="3" t="inlineStr">
@@ -33967,7 +33967,7 @@
           <t>Participación completa en el cuaderno simulado</t>
         </is>
       </c>
-      <c r="E106" s="4" t="n">
+      <c r="E106" s="6" t="n">
         <v>46322</v>
       </c>
       <c r="F106" s="3" t="inlineStr">
@@ -33995,7 +33995,7 @@
           <t>Participación completa en el cuaderno simulado</t>
         </is>
       </c>
-      <c r="E107" s="4" t="n">
+      <c r="E107" s="6" t="n">
         <v>46323</v>
       </c>
       <c r="F107" s="3" t="inlineStr">
@@ -34023,7 +34023,7 @@
           <t>Participación completa en el cuaderno simulado</t>
         </is>
       </c>
-      <c r="E108" s="4" t="n">
+      <c r="E108" s="6" t="n">
         <v>46325</v>
       </c>
       <c r="F108" s="3" t="inlineStr">
@@ -34051,7 +34051,7 @@
           <t>Participación completa en el cuaderno simulado</t>
         </is>
       </c>
-      <c r="E109" s="4" t="n">
+      <c r="E109" s="6" t="n">
         <v>46324</v>
       </c>
       <c r="F109" s="3" t="inlineStr">
@@ -34079,7 +34079,7 @@
           <t>Participación completa en el cuaderno simulado</t>
         </is>
       </c>
-      <c r="E110" s="4" t="n">
+      <c r="E110" s="6" t="n">
         <v>46322</v>
       </c>
       <c r="F110" s="3" t="inlineStr">
@@ -34107,7 +34107,7 @@
           <t>Participación completa en el cuaderno simulado</t>
         </is>
       </c>
-      <c r="E111" s="4" t="n">
+      <c r="E111" s="6" t="n">
         <v>46324</v>
       </c>
       <c r="F111" s="3" t="inlineStr">
@@ -34135,7 +34135,7 @@
           <t>Participación completa en el cuaderno simulado</t>
         </is>
       </c>
-      <c r="E112" s="4" t="n">
+      <c r="E112" s="6" t="n">
         <v>46323</v>
       </c>
       <c r="F112" s="3" t="inlineStr">

</xml_diff>